<commit_message>
feat(#479): added amPopCatchmentTotal column in optimization analysis
</commit_message>
<xml_diff>
--- a/tests/optimization/data/result_table.xlsx
+++ b/tests/optimization/data/result_table.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -367,10 +367,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>amPopCatchmentTotal</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>amPopCovered</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>amPopCoveredCumul</t>
         </is>
@@ -384,10 +389,13 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>1863123.143259477</v>
+        <v>1863123.125</v>
       </c>
       <c r="D2">
-        <v>1863123.143259477</v>
+        <v>1863123.125</v>
+      </c>
+      <c r="E2">
+        <v>1863123.125</v>
       </c>
     </row>
     <row r="3">
@@ -398,10 +406,13 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>84799.26954790266</v>
+        <v>1376554.875</v>
       </c>
       <c r="D3">
-        <v>1947922.41280738</v>
+        <v>84799.2734375</v>
+      </c>
+      <c r="E3">
+        <v>1947922.3984375</v>
       </c>
     </row>
     <row r="4">
@@ -412,10 +423,13 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>50165.96088150261</v>
+        <v>1831583.75</v>
       </c>
       <c r="D4">
-        <v>1998088.373688883</v>
+        <v>50165.9609375</v>
+      </c>
+      <c r="E4">
+        <v>1998088.359375</v>
       </c>
     </row>
     <row r="5">
@@ -426,10 +440,13 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <v>14928.8158991878</v>
+        <v>745185.875</v>
       </c>
       <c r="D5">
-        <v>2013017.18958807</v>
+        <v>14928.81640625</v>
+      </c>
+      <c r="E5">
+        <v>2013017.17578125</v>
       </c>
     </row>
     <row r="6">
@@ -440,10 +457,13 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>8129.587576460402</v>
+        <v>1594664.25</v>
       </c>
       <c r="D6">
-        <v>2021146.777164531</v>
+        <v>8129.58740234375</v>
+      </c>
+      <c r="E6">
+        <v>2021146.763183594</v>
       </c>
     </row>
     <row r="7">
@@ -454,10 +474,13 @@
         <v>9</v>
       </c>
       <c r="C7">
-        <v>6149.941541240893</v>
+        <v>1099307</v>
       </c>
       <c r="D7">
-        <v>2027296.718705772</v>
+        <v>6149.94140625</v>
+      </c>
+      <c r="E7">
+        <v>2027296.704589844</v>
       </c>
     </row>
     <row r="8">
@@ -468,10 +491,13 @@
         <v>3</v>
       </c>
       <c r="C8">
-        <v>6032.978334142325</v>
+        <v>6032.978515625</v>
       </c>
       <c r="D8">
-        <v>2033329.697039914</v>
+        <v>6032.978515625</v>
+      </c>
+      <c r="E8">
+        <v>2033329.683105469</v>
       </c>
     </row>
     <row r="9">
@@ -482,10 +508,13 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>3751.705136057301</v>
+        <v>3751.705078125</v>
       </c>
       <c r="D9">
-        <v>2037081.402175971</v>
+        <v>3751.705078125</v>
+      </c>
+      <c r="E9">
+        <v>2037081.388183594</v>
       </c>
     </row>
     <row r="10">
@@ -496,10 +525,13 @@
         <v>1</v>
       </c>
       <c r="C10">
-        <v>2513.095166622566</v>
+        <v>2513.09521484375</v>
       </c>
       <c r="D10">
-        <v>2039594.497342594</v>
+        <v>2513.09521484375</v>
+      </c>
+      <c r="E10">
+        <v>2039594.483398438</v>
       </c>
     </row>
     <row r="11">
@@ -510,10 +542,13 @@
         <v>10</v>
       </c>
       <c r="C11">
+        <v>96641.609375</v>
+      </c>
+      <c r="D11">
         <v>0</v>
       </c>
-      <c r="D11">
-        <v>2039594.497342594</v>
+      <c r="E11">
+        <v>2039594.483398438</v>
       </c>
     </row>
   </sheetData>

</xml_diff>